<commit_message>
3.12.11 Atualizada a exibição do tempo alvo nos processos para incluir formatação condicional e adicionado arquivo temporário de planilha.
</commit_message>
<xml_diff>
--- a/Documentos/Peças dos Estampos - CRASHFORM.xlsx
+++ b/Documentos/Peças dos Estampos - CRASHFORM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FERRAMENTARIA\Documents\GESTAO_FERRAMENTARIA\Documentos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fabio Bitencourt\Desktop\GESTÃO_FERRAMENTARIA\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D300DD2-10CE-4BB5-8321-AC8D430E86C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20831F9E-B958-49B1-9985-C8367BF326CA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Peças" sheetId="1" r:id="rId1"/>
@@ -21,17 +21,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
     </ext>
@@ -40,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="71">
   <si>
     <t>estampo_id</t>
   </si>
@@ -139,6 +128,120 @@
   </si>
   <si>
     <t>Punção Postiço</t>
+  </si>
+  <si>
+    <t>peca_id</t>
+  </si>
+  <si>
+    <t>nome_operacao</t>
+  </si>
+  <si>
+    <t>ordem_execucao</t>
+  </si>
+  <si>
+    <t>maquina_sugerida</t>
+  </si>
+  <si>
+    <t>tempo_estimado_horas</t>
+  </si>
+  <si>
+    <t>SELECT</t>
+  </si>
+  <si>
+    <t>Desmontar Porta Estampo</t>
+  </si>
+  <si>
+    <t>Bancada de Ferramentas</t>
+  </si>
+  <si>
+    <t>Bancada de Ferramentas, Pórtico</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>Banco</t>
+  </si>
+  <si>
+    <t>Programação CNC</t>
+  </si>
+  <si>
+    <t>Software CAM</t>
+  </si>
+  <si>
+    <t>8.0</t>
+  </si>
+  <si>
+    <t>Fresamento CNC</t>
+  </si>
+  <si>
+    <t>Centro de Usinagem</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>4.0</t>
+  </si>
+  <si>
+    <t>2.0</t>
+  </si>
+  <si>
+    <t>Rebarbação e Usinagem das Roscas</t>
+  </si>
+  <si>
+    <t>Bancada de Ferramentas e Furadeira de Coluna</t>
+  </si>
+  <si>
+    <t>Montagem das Colunas Guias</t>
+  </si>
+  <si>
+    <t>Montagem das Buchas Guias</t>
+  </si>
+  <si>
+    <t>Verificar Material</t>
+  </si>
+  <si>
+    <t>0.25</t>
+  </si>
+  <si>
+    <t>Torneamento</t>
+  </si>
+  <si>
+    <t>Torno Convencional</t>
+  </si>
+  <si>
+    <t>Retificação</t>
+  </si>
+  <si>
+    <t>Retífica Plana</t>
+  </si>
+  <si>
+    <t>3.0</t>
+  </si>
+  <si>
+    <t>1.5</t>
+  </si>
+  <si>
+    <t>Controle Dimensional</t>
+  </si>
+  <si>
+    <t>Fresamento Convencional</t>
+  </si>
+  <si>
+    <t>Fresadora Universal</t>
+  </si>
+  <si>
+    <t>Retíficação</t>
+  </si>
+  <si>
+    <t>Corte dos perfis</t>
+  </si>
+  <si>
+    <t>Eletroerosão a fio</t>
+  </si>
+  <si>
+    <t>Rebarbação</t>
   </si>
 </sst>
 </file>
@@ -173,7 +276,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -196,21 +299,263 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -229,9 +574,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -269,7 +614,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -375,7 +720,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -517,7 +862,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -561,22 +906,22 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5">
+      <c r="A2" s="1">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="3">
         <v>4</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G2" t="str">
@@ -585,22 +930,22 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5">
+      <c r="A3" s="1">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G3" t="str">
@@ -609,22 +954,22 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5">
-        <v>3</v>
-      </c>
-      <c r="C4" s="5">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G4" t="str">
@@ -633,22 +978,22 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3">
         <v>4</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <v>1</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G5" t="str">
@@ -657,22 +1002,22 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3">
         <v>5</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="3">
         <v>4</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G6" t="str">
@@ -681,22 +1026,22 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5">
+      <c r="A7" s="1">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3">
         <v>6</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="3">
         <v>4</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G7" t="str">
@@ -705,22 +1050,22 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5">
+      <c r="A8" s="1">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3">
         <v>8</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="3">
         <v>1</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G8" t="str">
@@ -729,22 +1074,22 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
-        <v>3</v>
-      </c>
-      <c r="B9" s="5">
+      <c r="A9" s="1">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3">
         <v>9</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="3">
         <v>1</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G9" t="str">
@@ -753,22 +1098,22 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="3">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5">
+      <c r="A10" s="1">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3">
         <v>10</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="3">
         <v>1</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G10" t="str">
@@ -777,22 +1122,22 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5">
+      <c r="A11" s="1">
+        <v>3</v>
+      </c>
+      <c r="B11" s="3">
         <v>11</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="3">
         <v>1</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G11" t="str">
@@ -801,22 +1146,22 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
-        <v>3</v>
-      </c>
-      <c r="B12" s="5">
+      <c r="A12" s="1">
+        <v>3</v>
+      </c>
+      <c r="B12" s="3">
         <v>12</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="3">
         <v>1</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G12" t="str">
@@ -825,22 +1170,22 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="3">
-        <v>3</v>
-      </c>
-      <c r="B13" s="5">
+      <c r="A13" s="1">
+        <v>3</v>
+      </c>
+      <c r="B13" s="3">
         <v>13</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="3">
         <v>1</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G13" t="str">
@@ -849,22 +1194,22 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="3">
-        <v>3</v>
-      </c>
-      <c r="B14" s="5">
+      <c r="A14" s="1">
+        <v>3</v>
+      </c>
+      <c r="B14" s="3">
         <v>14</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="3">
         <v>1</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G14" t="str">
@@ -873,22 +1218,22 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="3">
-        <v>3</v>
-      </c>
-      <c r="B15" s="5">
+      <c r="A15" s="1">
+        <v>3</v>
+      </c>
+      <c r="B15" s="3">
         <v>15</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="3">
         <v>1</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G15" t="str">
@@ -897,22 +1242,22 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="3">
-        <v>3</v>
-      </c>
-      <c r="B16" s="5">
+      <c r="A16" s="1">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3">
         <v>16</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="3">
         <v>1</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G16" t="str">
@@ -921,22 +1266,22 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="3">
-        <v>3</v>
-      </c>
-      <c r="B17" s="5">
+      <c r="A17" s="1">
+        <v>3</v>
+      </c>
+      <c r="B17" s="3">
         <v>17</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="3">
         <v>1</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G17" t="str">
@@ -945,22 +1290,22 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="3">
-        <v>3</v>
-      </c>
-      <c r="B18" s="5">
+      <c r="A18" s="1">
+        <v>3</v>
+      </c>
+      <c r="B18" s="3">
         <v>18</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="3">
         <v>1</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G18" t="str">
@@ -969,22 +1314,22 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="3">
-        <v>3</v>
-      </c>
-      <c r="B19" s="5">
+      <c r="A19" s="1">
+        <v>3</v>
+      </c>
+      <c r="B19" s="3">
         <v>19</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="3">
         <v>1</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G19" t="str">
@@ -993,22 +1338,22 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="3">
-        <v>3</v>
-      </c>
-      <c r="B20" s="5">
+      <c r="A20" s="1">
+        <v>3</v>
+      </c>
+      <c r="B20" s="3">
         <v>20</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="3">
         <v>4</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G20" t="str">
@@ -1017,22 +1362,22 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="3">
-        <v>3</v>
-      </c>
-      <c r="B21" s="5">
+      <c r="A21" s="1">
+        <v>3</v>
+      </c>
+      <c r="B21" s="3">
         <v>47</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="3">
         <v>1</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G21" t="str">
@@ -1041,22 +1386,22 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="3">
-        <v>3</v>
-      </c>
-      <c r="B22" s="5">
+      <c r="A22" s="1">
+        <v>3</v>
+      </c>
+      <c r="B22" s="3">
         <v>51</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="3">
         <v>4</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G22" t="str">
@@ -1071,21 +1416,616 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C991F7F8-3358-49FF-A4C6-92E8667CB718}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="61" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86" customWidth="1"/>
+    <col min="2" max="2" width="8" hidden="1" customWidth="1"/>
+    <col min="3" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="168.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D13&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16">
+        <v>1</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="17" t="str">
+        <f>"("&amp;A2&amp;""&amp;B2&amp;","&amp;"'"&amp;C2&amp;"'"&amp;","&amp;"'"&amp;D2&amp;"'"&amp;","&amp;"'"&amp;E2&amp;"'"&amp;","&amp;"'"&amp;F2&amp;"'"&amp;")"&amp;","</f>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1),'1','Desmontar Porta Estampo','Bancada de Ferramentas, Pórtico','1.0'),</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D13&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="9" t="str">
+        <f t="shared" ref="G3:G30" si="0">"("&amp;A3&amp;""&amp;B3&amp;","&amp;"'"&amp;C3&amp;"'"&amp;","&amp;"'"&amp;D3&amp;"'"&amp;","&amp;"'"&amp;E3&amp;"'"&amp;","&amp;"'"&amp;F3&amp;"'"&amp;")"&amp;","</f>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1),'2','Programação CNC','Software CAM','8.0'),</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D13&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1),'3','Fresamento CNC','Centro de Usinagem','10.0'),</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D13&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4">
+        <v>4</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1),'4','Rebarbação e Usinagem das Roscas','Bancada de Ferramentas e Furadeira de Coluna','4.0'),</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D13&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11">
+        <v>5</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Base Superior' AND estampo_id = 3 LIMIT 1),'5','Montagem das Colunas Guias','Bancada de Ferramentas','2.0'),</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D14&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1),'1','Desmontar Porta Estampo','Bancada de Ferramentas, Pórtico','1.0'),</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D14&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1),'2','Programação CNC','Software CAM','8.0'),</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D14&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4">
+        <v>3</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1),'3','Fresamento CNC','Centro de Usinagem','10.0'),</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D14&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4">
+        <v>4</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1),'4','Rebarbação e Usinagem das Roscas','Bancada de Ferramentas e Furadeira de Coluna','4.0'),</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="10" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D14&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11">
+        <v>5</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Placa Flutuante' AND estampo_id = 3 LIMIT 1),'5','Montagem das Buchas Guias','Bancada de Ferramentas','2.0'),</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D2&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1),'1','Verificar Material','Bancada de Ferramentas','0.25'),</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D2&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G15" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1),'2','Torneamento','Torno Convencional','3.0'),</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D2&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4">
+        <v>3</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1),'3','Retificação','Retífica Plana','1.5'),</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="10" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D2&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11">
+        <v>4</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G17" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Batente Estabilizador-Ø 31,8 x 71,2' AND estampo_id = 3 LIMIT 1),'4','Controle Dimensional','Bancada de Ferramentas','0.25'),</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D3&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G19" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1),'1','Verificar Material','Bancada de Ferramentas','0.25'),</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D3&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1),'2','Programação CNC','Software CAM','1.5'),</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D3&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4">
+        <v>3</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1),'3','Fresamento CNC','Centro de Usinagem','4.0'),</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D3&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4">
+        <v>4</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G22" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1),'4','Rebarbação e Usinagem das Roscas','Bancada de Ferramentas e Furadeira de Coluna','1.0'),</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="10" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D3&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11">
+        <v>5</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G23" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Garra 28 x 40 x 190' AND estampo_id = 3 LIMIT 1),'5','Controle Dimensional','Bancada de Ferramentas','0.25'),</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D4&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G25" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1),'1','Verificar Material','Bancada de Ferramentas','0.25'),</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D4&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4">
+        <v>2</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G26" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1),'2','Programação CNC','Software CAM','1.5'),</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D4&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4">
+        <v>3</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G27" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1),'3','Fresamento Convencional','Fresadora Universal','1.5'),</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D4&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4">
+        <v>4</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G28" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1),'4','Retíficação','Retífica Plana','1.5'),</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="8" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D4&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4">
+        <v>5</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G29" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1),'5','Corte dos perfis','Eletroerosão a fio','3.0'),</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="10" t="str">
+        <f>"(SELECT id FROM pecas WHERE nome = '"&amp;Peças!D4&amp;"' AND estampo_id = 3 LIMIT 1)"</f>
+        <v>(SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1)</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11">
+        <v>6</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G30" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>((SELECT id FROM pecas WHERE nome = 'Guia Blank' AND estampo_id = 3 LIMIT 1),'6','Rebarbação','Bancada de Ferramentas','1.5'),</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>